<commit_message>
Created Initial Launch Test
Set Manual Tests project to save in 2021
Created Remove Icon Editor Settings.vi to help facillitate testing
</commit_message>
<xml_diff>
--- a/Test/Manual Tests/Reference Files/OTE_Icon Editor G-based_-- All --_-- All --.xlsx
+++ b/Test/Manual Tests/Reference Files/OTE_Icon Editor G-based_-- All --_-- All --.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\J63553\Projects\_LabVIEW Community\labview-icon-editor\Test\Manual Tests\Reference Files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5AEBDDD7-EEE1-4E79-93D6-717C9444E99D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FCFF632-B477-43CE-A7A4-704E8514BB29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="85">
   <si>
     <t>TestCaseId</t>
   </si>
@@ -368,7 +368,10 @@
     <t>Test Procedure</t>
   </si>
   <si>
-    <t>01 Launch Test</t>
+    <t>02 Launch Test</t>
+  </si>
+  <si>
+    <t>01 Initial Launch Test</t>
   </si>
 </sst>
 </file>
@@ -829,22 +832,24 @@
       </c>
     </row>
     <row r="2" spans="1:6" ht="189" x14ac:dyDescent="0.25">
-      <c r="A2" s="7">
+      <c r="A2" s="8">
         <v>1692474</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="C2" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="D2" s="7" t="s">
+      <c r="D2" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="E2" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="F2" s="4"/>
+      <c r="E2" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>84</v>
+      </c>
     </row>
     <row r="3" spans="1:6" ht="110.25" x14ac:dyDescent="0.25">
       <c r="A3" s="7">
@@ -1306,23 +1311,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="5b2a8b02-cd78-409b-af2d-4bd8301a3454" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101006E386811B48EF74FB47FB32804B330A0" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="9605319a87d107f99f8e3a474ee978dd">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="5b2a8b02-cd78-409b-af2d-4bd8301a3454" xmlns:ns4="d752a718-7967-4073-bd35-1eb9c09a9d9e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="684eab0a72efee18062b2c121d46ea94" ns3:_="" ns4:_="">
     <xsd:import namespace="5b2a8b02-cd78-409b-af2d-4bd8301a3454"/>
@@ -1561,32 +1549,24 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FF6FFCCF-ABB3-4E35-8127-461338974DF1}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="d752a718-7967-4073-bd35-1eb9c09a9d9e"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="5b2a8b02-cd78-409b-af2d-4bd8301a3454"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6B930B2B-2F39-4180-93B5-1286877B435F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="5b2a8b02-cd78-409b-af2d-4bd8301a3454" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{82827F01-413F-4F6B-9442-EE2D35EBC2A7}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1603,4 +1583,29 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6B930B2B-2F39-4180-93B5-1286877B435F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FF6FFCCF-ABB3-4E35-8127-461338974DF1}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="d752a718-7967-4073-bd35-1eb9c09a9d9e"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="5b2a8b02-cd78-409b-af2d-4bd8301a3454"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Created 04 Glyphs test
</commit_message>
<xml_diff>
--- a/Test/Manual Tests/Reference Files/OTE_Icon Editor G-based_-- All --_-- All --.xlsx
+++ b/Test/Manual Tests/Reference Files/OTE_Icon Editor G-based_-- All --_-- All --.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\J63553\Projects\_LabVIEW Community\labview-icon-editor\Test\Manual Tests\Reference Files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{743BAD2B-7135-41F9-A34F-26D9F2A174B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC824B84-F92E-48E3-B788-A89FFD084AEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="95">
   <si>
     <t>TestCaseId</t>
   </si>
@@ -365,22 +365,10 @@
     <t>03 Templates</t>
   </si>
   <si>
-    <t>Saving of templates in 03 Templates
-Saving of glyphs still to be implemented.</t>
-  </si>
-  <si>
-    <t>Template names in 03 Templates
-Glyph names still to be implemented</t>
-  </si>
-  <si>
     <t>Is this actually IE related?
 Are these functions using the API?</t>
   </si>
   <si>
-    <t>Template search in 03 Templates
-Glyph search still to be implemented</t>
-  </si>
-  <si>
     <t>These steps are covered in other tests
 May be worth having a "quick" test to go through when reviewing PRs</t>
   </si>
@@ -390,6 +378,14 @@
   </si>
   <si>
     <t>These steps are covered in other tests. No need to create another test from this.</t>
+  </si>
+  <si>
+    <t>Saving of templates in 03 Templates
+Saving of glyphs in 04 Glyphs.</t>
+  </si>
+  <si>
+    <t>Template names in 03 Templates
+Glyph names in 04 Glyphs</t>
   </si>
 </sst>
 </file>
@@ -1009,26 +1005,26 @@
       <c r="G5" s="12"/>
     </row>
     <row r="6" spans="1:7" ht="150" x14ac:dyDescent="0.25">
-      <c r="A6" s="17">
+      <c r="A6" s="9">
         <v>1692479</v>
       </c>
-      <c r="B6" s="17" t="s">
+      <c r="B6" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="C6" s="18" t="s">
+      <c r="C6" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="D6" s="17" t="s">
+      <c r="D6" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="E6" s="17" t="s">
-        <v>8</v>
-      </c>
-      <c r="F6" s="19" t="s">
+      <c r="E6" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="F6" s="11" t="s">
         <v>88</v>
       </c>
-      <c r="G6" s="20" t="s">
-        <v>89</v>
+      <c r="G6" s="12" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="300" x14ac:dyDescent="0.25">
@@ -1070,26 +1066,26 @@
       <c r="G8" s="16"/>
     </row>
     <row r="9" spans="1:7" ht="75" x14ac:dyDescent="0.25">
-      <c r="A9" s="17">
+      <c r="A9" s="9">
         <v>1692483</v>
       </c>
-      <c r="B9" s="17" t="s">
+      <c r="B9" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="C9" s="18" t="s">
+      <c r="C9" s="10" t="s">
         <v>74</v>
       </c>
-      <c r="D9" s="17" t="s">
+      <c r="D9" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="E9" s="17" t="s">
-        <v>8</v>
-      </c>
-      <c r="F9" s="19" t="s">
+      <c r="E9" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="F9" s="11" t="s">
         <v>88</v>
       </c>
-      <c r="G9" s="20" t="s">
-        <v>90</v>
+      <c r="G9" s="12" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="165" x14ac:dyDescent="0.25">
@@ -1224,30 +1220,30 @@
       </c>
       <c r="F16" s="15"/>
       <c r="G16" s="16" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="135" x14ac:dyDescent="0.25">
-      <c r="A17" s="17">
+      <c r="A17" s="9">
         <v>1692493</v>
       </c>
-      <c r="B17" s="17" t="s">
+      <c r="B17" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="C17" s="18" t="s">
+      <c r="C17" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="D17" s="17" t="s">
+      <c r="D17" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="E17" s="17" t="s">
-        <v>8</v>
-      </c>
-      <c r="F17" s="19" t="s">
+      <c r="E17" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="F17" s="11" t="s">
         <v>88</v>
       </c>
-      <c r="G17" s="20" t="s">
-        <v>92</v>
+      <c r="G17" s="12" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="60" x14ac:dyDescent="0.25">
@@ -1346,7 +1342,7 @@
         <v>88</v>
       </c>
       <c r="G22" s="20" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="360" x14ac:dyDescent="0.25">
@@ -1366,10 +1362,10 @@
         <v>8</v>
       </c>
       <c r="F23" s="19" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="G23" s="20" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="70.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1411,7 +1407,7 @@
         <v>63</v>
       </c>
       <c r="G25" s="20" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
     </row>
     <row r="26" spans="1:7" ht="30" x14ac:dyDescent="0.25">
@@ -1457,6 +1453,23 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="5b2a8b02-cd78-409b-af2d-4bd8301a3454" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101006E386811B48EF74FB47FB32804B330A0" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="9605319a87d107f99f8e3a474ee978dd">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="5b2a8b02-cd78-409b-af2d-4bd8301a3454" xmlns:ns4="d752a718-7967-4073-bd35-1eb9c09a9d9e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="684eab0a72efee18062b2c121d46ea94" ns3:_="" ns4:_="">
     <xsd:import namespace="5b2a8b02-cd78-409b-af2d-4bd8301a3454"/>
@@ -1695,24 +1708,32 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FF6FFCCF-ABB3-4E35-8127-461338974DF1}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="d752a718-7967-4073-bd35-1eb9c09a9d9e"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="5b2a8b02-cd78-409b-af2d-4bd8301a3454"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="5b2a8b02-cd78-409b-af2d-4bd8301a3454" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6B930B2B-2F39-4180-93B5-1286877B435F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{82827F01-413F-4F6B-9442-EE2D35EBC2A7}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1729,29 +1750,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6B930B2B-2F39-4180-93B5-1286877B435F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FF6FFCCF-ABB3-4E35-8127-461338974DF1}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="d752a718-7967-4073-bd35-1eb9c09a9d9e"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="5b2a8b02-cd78-409b-af2d-4bd8301a3454"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Corrections to 04 Glyphs test
Added tests that were missed in the first pass
</commit_message>
<xml_diff>
--- a/Test/Manual Tests/Reference Files/OTE_Icon Editor G-based_-- All --_-- All --.xlsx
+++ b/Test/Manual Tests/Reference Files/OTE_Icon Editor G-based_-- All --_-- All --.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\J63553\Projects\_LabVIEW Community\labview-icon-editor\Test\Manual Tests\Reference Files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC824B84-F92E-48E3-B788-A89FFD084AEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77BFA199-B936-4846-A05C-7121E8BD611E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="98">
   <si>
     <t>TestCaseId</t>
   </si>
@@ -386,6 +386,16 @@
   <si>
     <t>Template names in 03 Templates
 Glyph names in 04 Glyphs</t>
+  </si>
+  <si>
+    <t>04 Glyphs</t>
+  </si>
+  <si>
+    <t>Need to test with no connection</t>
+  </si>
+  <si>
+    <t>03 Templates
+04 Glyphs</t>
   </si>
 </sst>
 </file>
@@ -1021,7 +1031,7 @@
         <v>8</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>88</v>
+        <v>97</v>
       </c>
       <c r="G6" s="12" t="s">
         <v>93</v>
@@ -1047,23 +1057,25 @@
       <c r="G7" s="16"/>
     </row>
     <row r="8" spans="1:7" ht="195" x14ac:dyDescent="0.25">
-      <c r="A8" s="13">
+      <c r="A8" s="9">
         <v>1692481</v>
       </c>
-      <c r="B8" s="13" t="s">
+      <c r="B8" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="C8" s="14" t="s">
+      <c r="C8" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="D8" s="13" t="s">
+      <c r="D8" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="E8" s="13" t="s">
-        <v>8</v>
-      </c>
-      <c r="F8" s="15"/>
-      <c r="G8" s="16"/>
+      <c r="E8" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="F8" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="G8" s="12"/>
     </row>
     <row r="9" spans="1:7" ht="75" x14ac:dyDescent="0.25">
       <c r="A9" s="9">
@@ -1082,7 +1094,7 @@
         <v>8</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>88</v>
+        <v>97</v>
       </c>
       <c r="G9" s="12" t="s">
         <v>94</v>
@@ -1165,23 +1177,25 @@
       <c r="G13" s="24"/>
     </row>
     <row r="14" spans="1:7" ht="165" x14ac:dyDescent="0.25">
-      <c r="A14" s="13">
+      <c r="A14" s="9">
         <v>1692490</v>
       </c>
-      <c r="B14" s="13" t="s">
+      <c r="B14" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="C14" s="14" t="s">
+      <c r="C14" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="D14" s="13" t="s">
+      <c r="D14" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="E14" s="13" t="s">
-        <v>8</v>
-      </c>
-      <c r="F14" s="15"/>
-      <c r="G14" s="16"/>
+      <c r="E14" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="F14" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="G14" s="12"/>
     </row>
     <row r="15" spans="1:7" ht="60" x14ac:dyDescent="0.25">
       <c r="A15" s="13">
@@ -1247,23 +1261,25 @@
       </c>
     </row>
     <row r="18" spans="1:7" ht="60" x14ac:dyDescent="0.25">
-      <c r="A18" s="13">
+      <c r="A18" s="9">
         <v>1692494</v>
       </c>
-      <c r="B18" s="13" t="s">
+      <c r="B18" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="C18" s="14" t="s">
+      <c r="C18" s="10" t="s">
         <v>82</v>
       </c>
-      <c r="D18" s="13" t="s">
+      <c r="D18" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="E18" s="13" t="s">
-        <v>8</v>
-      </c>
-      <c r="F18" s="15"/>
-      <c r="G18" s="16"/>
+      <c r="E18" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="F18" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="G18" s="12"/>
     </row>
     <row r="19" spans="1:7" ht="150" x14ac:dyDescent="0.25">
       <c r="A19" s="13">
@@ -1411,23 +1427,27 @@
       </c>
     </row>
     <row r="26" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A26" s="13">
+      <c r="A26" s="9">
         <v>1692503</v>
       </c>
-      <c r="B26" s="13" t="s">
+      <c r="B26" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="C26" s="14" t="s">
+      <c r="C26" s="10" t="s">
         <v>87</v>
       </c>
-      <c r="D26" s="13" t="s">
+      <c r="D26" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="E26" s="13" t="s">
-        <v>8</v>
-      </c>
-      <c r="F26" s="15"/>
-      <c r="G26" s="16"/>
+      <c r="E26" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="F26" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="G26" s="12" t="s">
+        <v>96</v>
+      </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
@@ -1453,23 +1473,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="5b2a8b02-cd78-409b-af2d-4bd8301a3454" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101006E386811B48EF74FB47FB32804B330A0" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="9605319a87d107f99f8e3a474ee978dd">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="5b2a8b02-cd78-409b-af2d-4bd8301a3454" xmlns:ns4="d752a718-7967-4073-bd35-1eb9c09a9d9e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="684eab0a72efee18062b2c121d46ea94" ns3:_="" ns4:_="">
     <xsd:import namespace="5b2a8b02-cd78-409b-af2d-4bd8301a3454"/>
@@ -1708,32 +1711,24 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FF6FFCCF-ABB3-4E35-8127-461338974DF1}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="d752a718-7967-4073-bd35-1eb9c09a9d9e"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="5b2a8b02-cd78-409b-af2d-4bd8301a3454"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6B930B2B-2F39-4180-93B5-1286877B435F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="5b2a8b02-cd78-409b-af2d-4bd8301a3454" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{82827F01-413F-4F6B-9442-EE2D35EBC2A7}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1750,4 +1745,29 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6B930B2B-2F39-4180-93B5-1286877B435F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FF6FFCCF-ABB3-4E35-8127-461338974DF1}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="d752a718-7967-4073-bd35-1eb9c09a9d9e"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="5b2a8b02-cd78-409b-af2d-4bd8301a3454"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Started creating Layers test
</commit_message>
<xml_diff>
--- a/Test/Manual Tests/Reference Files/OTE_Icon Editor G-based_-- All --_-- All --.xlsx
+++ b/Test/Manual Tests/Reference Files/OTE_Icon Editor G-based_-- All --_-- All --.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\J63553\Projects\_LabVIEW Community\labview-icon-editor\Test\Manual Tests\Reference Files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77BFA199-B936-4846-A05C-7121E8BD611E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1E8CEA4-C386-4904-891C-86DABEA3E8BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="99">
   <si>
     <t>TestCaseId</t>
   </si>
@@ -396,6 +396,9 @@
   <si>
     <t>03 Templates
 04 Glyphs</t>
+  </si>
+  <si>
+    <t>06 Layers</t>
   </si>
 </sst>
 </file>
@@ -1100,7 +1103,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="165" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" ht="150" x14ac:dyDescent="0.25">
       <c r="A10" s="13">
         <v>1692484</v>
       </c>
@@ -1135,7 +1138,9 @@
       <c r="E11" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="F11" s="15"/>
+      <c r="F11" s="15" t="s">
+        <v>98</v>
+      </c>
       <c r="G11" s="16"/>
     </row>
     <row r="12" spans="1:7" ht="135" x14ac:dyDescent="0.25">
@@ -1281,7 +1286,7 @@
       </c>
       <c r="G18" s="12"/>
     </row>
-    <row r="19" spans="1:7" ht="150" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" ht="135" x14ac:dyDescent="0.25">
       <c r="A19" s="13">
         <v>1692495</v>
       </c>
@@ -1316,10 +1321,12 @@
       <c r="E20" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="F20" s="15"/>
+      <c r="F20" s="15" t="s">
+        <v>98</v>
+      </c>
       <c r="G20" s="16"/>
     </row>
-    <row r="21" spans="1:7" ht="375" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" ht="360" x14ac:dyDescent="0.25">
       <c r="A21" s="13">
         <v>1692497</v>
       </c>
@@ -1361,7 +1368,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="23" spans="1:7" ht="360" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" ht="345" x14ac:dyDescent="0.25">
       <c r="A23" s="17">
         <v>1692499</v>
       </c>
@@ -1427,25 +1434,25 @@
       </c>
     </row>
     <row r="26" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A26" s="9">
+      <c r="A26" s="17">
         <v>1692503</v>
       </c>
-      <c r="B26" s="9" t="s">
+      <c r="B26" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="C26" s="10" t="s">
+      <c r="C26" s="18" t="s">
         <v>87</v>
       </c>
-      <c r="D26" s="9" t="s">
+      <c r="D26" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="E26" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="F26" s="11" t="s">
+      <c r="E26" s="17" t="s">
+        <v>8</v>
+      </c>
+      <c r="F26" s="19" t="s">
         <v>95</v>
       </c>
-      <c r="G26" s="12" t="s">
+      <c r="G26" s="20" t="s">
         <v>96</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Started development of Tools test
</commit_message>
<xml_diff>
--- a/Test/Manual Tests/Reference Files/OTE_Icon Editor G-based_-- All --_-- All --.xlsx
+++ b/Test/Manual Tests/Reference Files/OTE_Icon Editor G-based_-- All --_-- All --.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\J63553\Projects\_LabVIEW Community\labview-icon-editor\Test\Manual Tests\Reference Files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DE7FE2E-73F8-4404-AD8E-3A700DF54FE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDEF63A6-90F3-4F46-9EBA-866561F89DF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1996366;LabVIEW Master Test Pla" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="102">
   <si>
     <t>TestCaseId</t>
   </si>
@@ -407,6 +407,9 @@
   </si>
   <si>
     <t>Persistance Test</t>
+  </si>
+  <si>
+    <t>07 Tools</t>
   </si>
 </sst>
 </file>
@@ -1049,23 +1052,25 @@
       </c>
     </row>
     <row r="7" spans="1:7" ht="300" x14ac:dyDescent="0.25">
-      <c r="A7" s="13">
+      <c r="A7" s="17">
         <v>1692480</v>
       </c>
-      <c r="B7" s="13" t="s">
+      <c r="B7" s="17" t="s">
         <v>59</v>
       </c>
-      <c r="C7" s="14" t="s">
+      <c r="C7" s="18" t="s">
         <v>69</v>
       </c>
-      <c r="D7" s="13" t="s">
+      <c r="D7" s="17" t="s">
         <v>60</v>
       </c>
-      <c r="E7" s="13" t="s">
-        <v>8</v>
-      </c>
-      <c r="F7" s="15"/>
-      <c r="G7" s="16"/>
+      <c r="E7" s="17" t="s">
+        <v>8</v>
+      </c>
+      <c r="F7" s="19" t="s">
+        <v>101</v>
+      </c>
+      <c r="G7" s="20"/>
     </row>
     <row r="8" spans="1:7" ht="195" x14ac:dyDescent="0.25">
       <c r="A8" s="9">
@@ -1152,23 +1157,25 @@
       <c r="G11" s="16"/>
     </row>
     <row r="12" spans="1:7" ht="135" x14ac:dyDescent="0.25">
-      <c r="A12" s="13">
+      <c r="A12" s="17">
         <v>1692488</v>
       </c>
-      <c r="B12" s="13" t="s">
+      <c r="B12" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="C12" s="14" t="s">
+      <c r="C12" s="18" t="s">
         <v>77</v>
       </c>
-      <c r="D12" s="13" t="s">
+      <c r="D12" s="17" t="s">
         <v>45</v>
       </c>
-      <c r="E12" s="13" t="s">
-        <v>8</v>
-      </c>
-      <c r="F12" s="15"/>
-      <c r="G12" s="16"/>
+      <c r="E12" s="17" t="s">
+        <v>8</v>
+      </c>
+      <c r="F12" s="19" t="s">
+        <v>101</v>
+      </c>
+      <c r="G12" s="20"/>
     </row>
     <row r="13" spans="1:7" ht="240" x14ac:dyDescent="0.25">
       <c r="A13" s="21">
@@ -1490,23 +1497,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="5b2a8b02-cd78-409b-af2d-4bd8301a3454" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101006E386811B48EF74FB47FB32804B330A0" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="9605319a87d107f99f8e3a474ee978dd">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="5b2a8b02-cd78-409b-af2d-4bd8301a3454" xmlns:ns4="d752a718-7967-4073-bd35-1eb9c09a9d9e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="684eab0a72efee18062b2c121d46ea94" ns3:_="" ns4:_="">
     <xsd:import namespace="5b2a8b02-cd78-409b-af2d-4bd8301a3454"/>
@@ -1745,32 +1735,24 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FF6FFCCF-ABB3-4E35-8127-461338974DF1}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="d752a718-7967-4073-bd35-1eb9c09a9d9e"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="5b2a8b02-cd78-409b-af2d-4bd8301a3454"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6B930B2B-2F39-4180-93B5-1286877B435F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="5b2a8b02-cd78-409b-af2d-4bd8301a3454" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{82827F01-413F-4F6B-9442-EE2D35EBC2A7}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1787,4 +1769,29 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6B930B2B-2F39-4180-93B5-1286877B435F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FF6FFCCF-ABB3-4E35-8127-461338974DF1}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="d752a718-7967-4073-bd35-1eb9c09a9d9e"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="5b2a8b02-cd78-409b-af2d-4bd8301a3454"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>